<commit_message>
feat: add NotifyWizard, direct cellular SMS SIM and WhatsApp dispatch, student phone resolution
</commit_message>
<xml_diff>
--- a/backend/sample_files/IT_A_61_Students_Roster.xlsx
+++ b/backend/sample_files/IT_A_61_Students_Roster.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D61"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -418,10 +418,10 @@
         <v>922524205125</v>
       </c>
       <c r="B2" t="str">
-        <v>PRIYANKA M.K</v>
+        <v>Priyanka M.K</v>
       </c>
       <c r="C2" t="str">
-        <v>PRIYANKA M.K's Parent</v>
+        <v>Priyanka M.K's Parent</v>
       </c>
       <c r="D2" t="str">
         <v>8940915396</v>
@@ -432,10 +432,10 @@
         <v>922524205126</v>
       </c>
       <c r="B3" t="str">
-        <v>RAGUL R</v>
+        <v>Ragul R</v>
       </c>
       <c r="C3" t="str">
-        <v>RAGUL R's Parent</v>
+        <v>Ragul R's Parent</v>
       </c>
       <c r="D3" t="str">
         <v>6381598068</v>
@@ -446,10 +446,10 @@
         <v>922524205127</v>
       </c>
       <c r="B4" t="str">
-        <v>RAJASARANYA S</v>
+        <v>Rajasaranya S</v>
       </c>
       <c r="C4" t="str">
-        <v>RAJASARANYA S's Parent</v>
+        <v>Rajasaranya S's Parent</v>
       </c>
       <c r="D4" t="str">
         <v>7397021477</v>
@@ -460,10 +460,10 @@
         <v>922524205128</v>
       </c>
       <c r="B5" t="str">
-        <v>RAJAVARMAN R A</v>
+        <v>Rajavarman R A</v>
       </c>
       <c r="C5" t="str">
-        <v>RAJAVARMAN R A's Parent</v>
+        <v>Rajavarman R A's Parent</v>
       </c>
       <c r="D5" t="str">
         <v>9789826387</v>
@@ -474,10 +474,10 @@
         <v>922524205129</v>
       </c>
       <c r="B6" t="str">
-        <v>RAMAKRISHNAN M</v>
+        <v>Ramakrishnan M</v>
       </c>
       <c r="C6" t="str">
-        <v>RAMAKRISHNAN M's Parent</v>
+        <v>Ramakrishnan M's Parent</v>
       </c>
       <c r="D6" t="str">
         <v>9025535278</v>
@@ -488,10 +488,10 @@
         <v>922524205130</v>
       </c>
       <c r="B7" t="str">
-        <v>RAMKISHORE SM</v>
+        <v>Ramkishore S.M</v>
       </c>
       <c r="C7" t="str">
-        <v>RAMKISHORE SM's Parent</v>
+        <v>Ramkishore S.M's Parent</v>
       </c>
       <c r="D7" t="str">
         <v>8778764551</v>
@@ -502,10 +502,10 @@
         <v>922524205131</v>
       </c>
       <c r="B8" t="str">
-        <v>RANJANIDEVI R</v>
+        <v>Ranjanidevi R</v>
       </c>
       <c r="C8" t="str">
-        <v>RANJANIDEVI R's Parent</v>
+        <v>Ranjanidevi R's Parent</v>
       </c>
       <c r="D8" t="str">
         <v>9360729633</v>
@@ -516,10 +516,10 @@
         <v>922524205132</v>
       </c>
       <c r="B9" t="str">
-        <v>RANJITH KUMAR S</v>
+        <v>Ranjith Kumar S</v>
       </c>
       <c r="C9" t="str">
-        <v>RANJITH KUMAR S's Parent</v>
+        <v>Ranjith Kumar S's Parent</v>
       </c>
       <c r="D9" t="str">
         <v>8056656387</v>
@@ -530,10 +530,10 @@
         <v>922524205133</v>
       </c>
       <c r="B10" t="str">
-        <v>RANKANAYAKI V</v>
+        <v>Rankanayaki V</v>
       </c>
       <c r="C10" t="str">
-        <v>RANKANAYAKI V's Parent</v>
+        <v>Rankanayaki V's Parent</v>
       </c>
       <c r="D10" t="str">
         <v>9655211440</v>
@@ -544,10 +544,10 @@
         <v>922524205134</v>
       </c>
       <c r="B11" t="str">
-        <v>RIFA NOWREEN NATHAR EM</v>
+        <v>Rifa Nowreen Nathar E.M</v>
       </c>
       <c r="C11" t="str">
-        <v>RIFA NOWREEN NATHAR EM's Parent</v>
+        <v>Rifa Nowreen Nathar E.M's Parent</v>
       </c>
       <c r="D11" t="str">
         <v>6381504697</v>
@@ -558,10 +558,10 @@
         <v>922524205135</v>
       </c>
       <c r="B12" t="str">
-        <v>RITHEESHVER G</v>
+        <v>Ritheeshver G</v>
       </c>
       <c r="C12" t="str">
-        <v>RITHEESHVER G's Parent</v>
+        <v>Ritheeshver G's Parent</v>
       </c>
       <c r="D12" t="str">
         <v>9597671107</v>
@@ -572,10 +572,10 @@
         <v>922524205136</v>
       </c>
       <c r="B13" t="str">
-        <v>ROHITHSHARMA M</v>
+        <v>Rohithsharma M</v>
       </c>
       <c r="C13" t="str">
-        <v>ROHITHSHARMA M's Parent</v>
+        <v>Rohithsharma M's Parent</v>
       </c>
       <c r="D13" t="str">
         <v>6374995334</v>
@@ -586,10 +586,10 @@
         <v>922524205137</v>
       </c>
       <c r="B14" t="str">
-        <v>ROSHAN SAFIHA B</v>
+        <v>Roshan Safiha B</v>
       </c>
       <c r="C14" t="str">
-        <v>ROSHAN SAFIHA B's Parent</v>
+        <v>Roshan Safiha B's Parent</v>
       </c>
       <c r="D14" t="str">
         <v>9597597426</v>
@@ -600,10 +600,10 @@
         <v>922524205138</v>
       </c>
       <c r="B15" t="str">
-        <v>SABARI VASAN S</v>
+        <v>Sabari Vasan S</v>
       </c>
       <c r="C15" t="str">
-        <v>SABARI VASAN S's Parent</v>
+        <v>Sabari Vasan S's Parent</v>
       </c>
       <c r="D15" t="str">
         <v>8015365439</v>
@@ -614,10 +614,10 @@
         <v>922524205139</v>
       </c>
       <c r="B16" t="str">
-        <v>SABITHA P</v>
+        <v>Sabitha P</v>
       </c>
       <c r="C16" t="str">
-        <v>SABITHA P's Parent</v>
+        <v>Sabitha P's Parent</v>
       </c>
       <c r="D16" t="str">
         <v>8778527209</v>
@@ -628,10 +628,10 @@
         <v>922524205140</v>
       </c>
       <c r="B17" t="str">
-        <v>SAKTHIVEL S</v>
+        <v>Sakthivel S</v>
       </c>
       <c r="C17" t="str">
-        <v>SAKTHIVEL S's Parent</v>
+        <v>Sakthivel S's Parent</v>
       </c>
       <c r="D17" t="str">
         <v>9442183290</v>
@@ -642,10 +642,10 @@
         <v>922524205141</v>
       </c>
       <c r="B18" t="str">
-        <v>SALETH JOSELA A</v>
+        <v>Saleth Josela A</v>
       </c>
       <c r="C18" t="str">
-        <v>SALETH JOSELA A's Parent</v>
+        <v>Saleth Josela A's Parent</v>
       </c>
       <c r="D18" t="str">
         <v>9790210183</v>
@@ -656,10 +656,10 @@
         <v>922524205142</v>
       </c>
       <c r="B19" t="str">
-        <v>SANJAY K</v>
+        <v>Sanjay K</v>
       </c>
       <c r="C19" t="str">
-        <v>SANJAY K's Parent</v>
+        <v>Sanjay K's Parent</v>
       </c>
       <c r="D19" t="str">
         <v>9345787220</v>
@@ -670,10 +670,10 @@
         <v>922524205143</v>
       </c>
       <c r="B20" t="str">
-        <v>SANJAY S</v>
+        <v>Sanjay S</v>
       </c>
       <c r="C20" t="str">
-        <v>SANJAY S's Parent</v>
+        <v>Sanjay S's Parent</v>
       </c>
       <c r="D20" t="str">
         <v>9489841868</v>
@@ -684,10 +684,10 @@
         <v>922524205144</v>
       </c>
       <c r="B21" t="str">
-        <v>SANJEEVANI M M</v>
+        <v>Sanjeevani M M</v>
       </c>
       <c r="C21" t="str">
-        <v>SANJEEVANI M M's Parent</v>
+        <v>Sanjeevani M M's Parent</v>
       </c>
       <c r="D21" t="str">
         <v>9003459989</v>
@@ -698,10 +698,10 @@
         <v>922524205145</v>
       </c>
       <c r="B22" t="str">
-        <v>SANTHIYA B K</v>
+        <v>Santhiya B K</v>
       </c>
       <c r="C22" t="str">
-        <v>SANTHIYA B K's Parent</v>
+        <v>Santhiya B K's Parent</v>
       </c>
       <c r="D22" t="str">
         <v>9080751908</v>
@@ -712,13 +712,13 @@
         <v>922524205146</v>
       </c>
       <c r="B23" t="str">
-        <v>SANTHOSH KUMAR R</v>
+        <v>Santhoshkumar R</v>
       </c>
       <c r="C23" t="str">
-        <v>SANTHOSH KUMAR R's Parent</v>
+        <v>Santhoshkumar R's Parent</v>
       </c>
       <c r="D23" t="str">
-        <v>8072752322</v>
+        <v>6383474523</v>
       </c>
     </row>
     <row r="24">
@@ -726,10 +726,10 @@
         <v>922524205147</v>
       </c>
       <c r="B24" t="str">
-        <v>SANTHOSH S</v>
+        <v>Santhosh S</v>
       </c>
       <c r="C24" t="str">
-        <v>SANTHOSH S's Parent</v>
+        <v>Santhosh S's Parent</v>
       </c>
       <c r="D24" t="str">
         <v>8807854679</v>
@@ -740,10 +740,10 @@
         <v>922524205148</v>
       </c>
       <c r="B25" t="str">
-        <v>SANTHOSHKUMAR S</v>
+        <v>Santhoshkumar S</v>
       </c>
       <c r="C25" t="str">
-        <v>SANTHOSHKUMAR S's Parent</v>
+        <v>Santhoshkumar S's Parent</v>
       </c>
       <c r="D25" t="str">
         <v>9487528706</v>
@@ -754,10 +754,10 @@
         <v>922524205149</v>
       </c>
       <c r="B26" t="str">
-        <v>SARAVANAN P</v>
+        <v>Saravanan P</v>
       </c>
       <c r="C26" t="str">
-        <v>SARAVANAN P's Parent</v>
+        <v>Saravanan P's Parent</v>
       </c>
       <c r="D26" t="str">
         <v>8072117461</v>
@@ -768,10 +768,10 @@
         <v>922524205150</v>
       </c>
       <c r="B27" t="str">
-        <v>SARMILA V</v>
+        <v>Sarmila V</v>
       </c>
       <c r="C27" t="str">
-        <v>SARMILA V's Parent</v>
+        <v>Sarmila V's Parent</v>
       </c>
       <c r="D27" t="str">
         <v>9344812750</v>
@@ -782,10 +782,10 @@
         <v>922524205151</v>
       </c>
       <c r="B28" t="str">
-        <v>SATHISH KUMAR P</v>
+        <v>Sathish Kumar P</v>
       </c>
       <c r="C28" t="str">
-        <v>SATHISH KUMAR P's Parent</v>
+        <v>Sathish Kumar P's Parent</v>
       </c>
       <c r="D28" t="str">
         <v>9345782544</v>
@@ -796,10 +796,10 @@
         <v>922524205152</v>
       </c>
       <c r="B29" t="str">
-        <v>SELVARAJ D</v>
+        <v>Selvaraj D</v>
       </c>
       <c r="C29" t="str">
-        <v>SELVARAJ D's Parent</v>
+        <v>Selvaraj D's Parent</v>
       </c>
       <c r="D29" t="str">
         <v>6381273534</v>
@@ -810,10 +810,10 @@
         <v>922524205153</v>
       </c>
       <c r="B30" t="str">
-        <v>SHARUPRAKASH P</v>
+        <v>Sharuprakash P</v>
       </c>
       <c r="C30" t="str">
-        <v>SHARUPRAKASH P's Parent</v>
+        <v>Sharuprakash P's Parent</v>
       </c>
       <c r="D30" t="str">
         <v>9363980381</v>
@@ -824,10 +824,10 @@
         <v>922524205154</v>
       </c>
       <c r="B31" t="str">
-        <v>SHRINITHI V</v>
+        <v>Shrinithi V</v>
       </c>
       <c r="C31" t="str">
-        <v>SHRINITHI V's Parent</v>
+        <v>Shrinithi V's Parent</v>
       </c>
       <c r="D31" t="str">
         <v>9159742474</v>
@@ -838,10 +838,10 @@
         <v>922524205155</v>
       </c>
       <c r="B32" t="str">
-        <v>SIVAPRASANTH S</v>
+        <v>Sivaprasanth S</v>
       </c>
       <c r="C32" t="str">
-        <v>SIVAPRASANTH S's Parent</v>
+        <v>Sivaprasanth S's Parent</v>
       </c>
       <c r="D32" t="str">
         <v>8248367978</v>
@@ -852,10 +852,10 @@
         <v>922524205156</v>
       </c>
       <c r="B33" t="str">
-        <v>SRIJANANI P</v>
+        <v>Srijanani P</v>
       </c>
       <c r="C33" t="str">
-        <v>SRIJANANI P's Parent</v>
+        <v>Srijanani P's Parent</v>
       </c>
       <c r="D33" t="str">
         <v>9363308718</v>
@@ -866,10 +866,10 @@
         <v>922524205157</v>
       </c>
       <c r="B34" t="str">
-        <v>SRINIDI R</v>
+        <v>Srinidi R</v>
       </c>
       <c r="C34" t="str">
-        <v>SRINIDI R's Parent</v>
+        <v>Srinidi R's Parent</v>
       </c>
       <c r="D34" t="str">
         <v>7708697023</v>
@@ -880,10 +880,10 @@
         <v>922524205159</v>
       </c>
       <c r="B35" t="str">
-        <v>SUJI M</v>
+        <v>Suji M</v>
       </c>
       <c r="C35" t="str">
-        <v>SUJI M's Parent</v>
+        <v>Suji M's Parent</v>
       </c>
       <c r="D35" t="str">
         <v>9344547989</v>
@@ -894,10 +894,10 @@
         <v>922524205160</v>
       </c>
       <c r="B36" t="str">
-        <v>SUJITH R</v>
+        <v>Sujith R</v>
       </c>
       <c r="C36" t="str">
-        <v>SUJITH R's Parent</v>
+        <v>Sujith R's Parent</v>
       </c>
       <c r="D36" t="str">
         <v>6385220810</v>
@@ -908,10 +908,10 @@
         <v>922524205161</v>
       </c>
       <c r="B37" t="str">
-        <v>SUPREYA M K</v>
+        <v>Supreya M K</v>
       </c>
       <c r="C37" t="str">
-        <v>SUPREYA M K's Parent</v>
+        <v>Supreya M K's Parent</v>
       </c>
       <c r="D37" t="str">
         <v>9655279272</v>
@@ -922,10 +922,10 @@
         <v>922524205162</v>
       </c>
       <c r="B38" t="str">
-        <v>SURIYAPRIYA V</v>
+        <v>Suriyapriya V</v>
       </c>
       <c r="C38" t="str">
-        <v>SURIYAPRIYA V's Parent</v>
+        <v>Suriyapriya V's Parent</v>
       </c>
       <c r="D38" t="str">
         <v>9597742637</v>
@@ -936,10 +936,10 @@
         <v>922524205163</v>
       </c>
       <c r="B39" t="str">
-        <v>SUVATHI N</v>
+        <v>Suvathi N</v>
       </c>
       <c r="C39" t="str">
-        <v>SUVATHI N's Parent</v>
+        <v>Suvathi N's Parent</v>
       </c>
       <c r="D39" t="str">
         <v>6369371391</v>
@@ -950,10 +950,10 @@
         <v>922524205164</v>
       </c>
       <c r="B40" t="str">
-        <v>SWATHI C</v>
+        <v>Swathi C</v>
       </c>
       <c r="C40" t="str">
-        <v>SWATHI C's Parent</v>
+        <v>Swathi C's Parent</v>
       </c>
       <c r="D40" t="str">
         <v>6380646845</v>
@@ -964,10 +964,10 @@
         <v>922524205165</v>
       </c>
       <c r="B41" t="str">
-        <v>SWATHI R</v>
+        <v>Swathi R</v>
       </c>
       <c r="C41" t="str">
-        <v>SWATHI R's Parent</v>
+        <v>Swathi R's Parent</v>
       </c>
       <c r="D41" t="str">
         <v>9363621521</v>
@@ -978,10 +978,10 @@
         <v>922524205166</v>
       </c>
       <c r="B42" t="str">
-        <v>SWETHAA V</v>
+        <v>Swethaa V</v>
       </c>
       <c r="C42" t="str">
-        <v>SWETHAA V's Parent</v>
+        <v>Swethaa V's Parent</v>
       </c>
       <c r="D42" t="str">
         <v>9080278197</v>
@@ -992,10 +992,10 @@
         <v>922524205167</v>
       </c>
       <c r="B43" t="str">
-        <v>TARUN KARTHICK G</v>
+        <v>Tarun Karthick G</v>
       </c>
       <c r="C43" t="str">
-        <v>TARUN KARTHICK G's Parent</v>
+        <v>Tarun Karthick G's Parent</v>
       </c>
       <c r="D43" t="str">
         <v>9788882442</v>
@@ -1006,10 +1006,10 @@
         <v>922524205168</v>
       </c>
       <c r="B44" t="str">
-        <v>THAMILNESAN I</v>
+        <v>Thamilnesan I</v>
       </c>
       <c r="C44" t="str">
-        <v>THAMILNESAN I's Parent</v>
+        <v>Thamilnesan I's Parent</v>
       </c>
       <c r="D44" t="str">
         <v>6383094190</v>
@@ -1017,259 +1017,245 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>922524205169</v>
+        <v>922524205170</v>
       </c>
       <c r="B45" t="str">
-        <v>THARANEESH D</v>
+        <v>Tharani T</v>
       </c>
       <c r="C45" t="str">
-        <v>THARANEESH D's Parent</v>
+        <v>Tharani T's Parent</v>
       </c>
       <c r="D45" t="str">
-        <v>9843406814</v>
+        <v>9500313240</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>922524205170</v>
+        <v>922524205171</v>
       </c>
       <c r="B46" t="str">
-        <v>THARANI T</v>
+        <v>Tharunkumar K</v>
       </c>
       <c r="C46" t="str">
-        <v>THARANI T's Parent</v>
+        <v>Tharunkumar K's Parent</v>
       </c>
       <c r="D46" t="str">
-        <v>9500313240</v>
+        <v>8760964830</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>922524205171</v>
+        <v>922524205172</v>
       </c>
       <c r="B47" t="str">
-        <v>THARUNKUMAR K</v>
+        <v>Theerthagiri J</v>
       </c>
       <c r="C47" t="str">
-        <v>THARUNKUMAR K's Parent</v>
+        <v>Theerthagiri J's Parent</v>
       </c>
       <c r="D47" t="str">
-        <v>8760964830</v>
+        <v>9159895331</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>922524205172</v>
+        <v>922524205173</v>
       </c>
       <c r="B48" t="str">
-        <v>THEERTHAGIRI J</v>
+        <v>Thiruvasagam V</v>
       </c>
       <c r="C48" t="str">
-        <v>THEERTHAGIRI J's Parent</v>
+        <v>Thiruvasagam V's Parent</v>
       </c>
       <c r="D48" t="str">
-        <v>9159895331</v>
+        <v>8248385411</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>922524205173</v>
+        <v>922524205174</v>
       </c>
       <c r="B49" t="str">
-        <v>THIRUVASAGAM V</v>
+        <v>Vanitha M</v>
       </c>
       <c r="C49" t="str">
-        <v>THIRUVASAGAM V's Parent</v>
+        <v>Vanitha M's Parent</v>
       </c>
       <c r="D49" t="str">
-        <v>8248385411</v>
+        <v>8610967540</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>922524205174</v>
+        <v>922524205175</v>
       </c>
       <c r="B50" t="str">
-        <v>VANITHA M</v>
+        <v>Varsha S</v>
       </c>
       <c r="C50" t="str">
-        <v>VANITHA M's Parent</v>
+        <v>Varsha S's Parent</v>
       </c>
       <c r="D50" t="str">
-        <v>8610967540</v>
+        <v>8610344144</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>922524205175</v>
+        <v>922524205176</v>
       </c>
       <c r="B51" t="str">
-        <v>VARSHA S</v>
+        <v>Varsheni T</v>
       </c>
       <c r="C51" t="str">
-        <v>VARSHA S's Parent</v>
+        <v>Varsheni T's Parent</v>
       </c>
       <c r="D51" t="str">
-        <v>8610344144</v>
+        <v>8838798298</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>922524205176</v>
+        <v>922524205177</v>
       </c>
       <c r="B52" t="str">
-        <v>VARSHENI T</v>
+        <v>Varshini S S</v>
       </c>
       <c r="C52" t="str">
-        <v>VARSHENI T's Parent</v>
+        <v>Varshini S S's Parent</v>
       </c>
       <c r="D52" t="str">
-        <v>8838798298</v>
+        <v>9486546552</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>922524205177</v>
+        <v>922524205178</v>
       </c>
       <c r="B53" t="str">
-        <v>VARSHINI S S</v>
+        <v>Vikash S</v>
       </c>
       <c r="C53" t="str">
-        <v>VARSHINI S S's Parent</v>
+        <v>Vikash S's Parent</v>
       </c>
       <c r="D53" t="str">
-        <v>9486546552</v>
+        <v>9345352504</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>922524205178</v>
+        <v>922524205179</v>
       </c>
       <c r="B54" t="str">
-        <v>VIKASH S</v>
+        <v>Vishalini B</v>
       </c>
       <c r="C54" t="str">
-        <v>VIKASH S's Parent</v>
+        <v>Vishalini B's Parent</v>
       </c>
       <c r="D54" t="str">
-        <v>9345352504</v>
+        <v>9488727640</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>922524205179</v>
+        <v>922524205180</v>
       </c>
       <c r="B55" t="str">
-        <v>VISHALINI B</v>
+        <v>Yamuna E</v>
       </c>
       <c r="C55" t="str">
-        <v>VISHALINI B's Parent</v>
+        <v>Yamuna E's Parent</v>
       </c>
       <c r="D55" t="str">
-        <v>9488727640</v>
+        <v>6380458603</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>922524205180</v>
+        <v>922524205181</v>
       </c>
       <c r="B56" t="str">
-        <v>YAMUNA E</v>
+        <v>Yogadharshini S</v>
       </c>
       <c r="C56" t="str">
-        <v>YAMUNA E's Parent</v>
+        <v>Yogadharshini S's Parent</v>
       </c>
       <c r="D56" t="str">
-        <v>6380458603</v>
+        <v>8248407545</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>922524205181</v>
+        <v>922524205182</v>
       </c>
       <c r="B57" t="str">
-        <v>YOGADHARSHINI S</v>
+        <v>Yogesh R</v>
       </c>
       <c r="C57" t="str">
-        <v>YOGADHARSHINI S's Parent</v>
+        <v>Yogesh R's Parent</v>
       </c>
       <c r="D57" t="str">
-        <v>8248407545</v>
+        <v>7339108816</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>922524205182</v>
+        <v>922524205183</v>
       </c>
       <c r="B58" t="str">
-        <v>YOGESH R</v>
+        <v>Yuvanesh P</v>
       </c>
       <c r="C58" t="str">
-        <v>YOGESH R's Parent</v>
+        <v>Yuvanesh P's Parent</v>
       </c>
       <c r="D58" t="str">
-        <v>7339108816</v>
+        <v>6379988358</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>922524205183</v>
+        <v>922524205184</v>
       </c>
       <c r="B59" t="str">
-        <v>YUVANESH P</v>
+        <v>Yuvansankar K</v>
       </c>
       <c r="C59" t="str">
-        <v>YUVANESH P's Parent</v>
+        <v>Yuvansankar K's Parent</v>
       </c>
       <c r="D59" t="str">
-        <v>6379988358</v>
+        <v>7904379985</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>922524205184</v>
+        <v>922524205185</v>
       </c>
       <c r="B60" t="str">
-        <v>YUVANSANKAR K</v>
+        <v>Srilekha S.C</v>
       </c>
       <c r="C60" t="str">
-        <v>YUVANSANKAR K's Parent</v>
+        <v>Srilekha S.C's Parent</v>
       </c>
       <c r="D60" t="str">
-        <v>7904379985</v>
+        <v>9789882471</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>922524205185</v>
+        <v>922524205303</v>
       </c>
       <c r="B61" t="str">
-        <v>SRILEKHA SC</v>
+        <v>Nadar Prakash Shivahakthivel S</v>
       </c>
       <c r="C61" t="str">
-        <v>SRILEKHA SC's Parent</v>
+        <v>Nadar Prakash Shivahakthivel S's Parent</v>
       </c>
       <c r="D61" t="str">
-        <v>9789882471</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>922524205303</v>
-      </c>
-      <c r="B62" t="str">
-        <v>NADAR PRAKASH SHIVAHAKTHIVEL S</v>
-      </c>
-      <c r="C62" t="str">
-        <v>NADAR PRAKASH SHIVAHAKTHIVEL S's Parent</v>
-      </c>
-      <c r="D62" t="str">
         <v>7710946257</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D61"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>